<commit_message>
changed some names of the colomns, the script was testes and it works well
</commit_message>
<xml_diff>
--- a/schuelerliste.xlsx
+++ b/schuelerliste.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ivan\Workspace\bg-school-certificate-generator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0222185C-952C-4137-B10B-D6F6C1F716D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54A15200-A4B5-4A32-A5CC-9A74331E7377}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10695" yWindow="3015" windowWidth="38700" windowHeight="15285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30" yWindow="135" windowWidth="51570" windowHeight="20850" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -25,19 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="34">
-  <si>
-    <t>Mitglied</t>
-  </si>
-  <si>
-    <t>Kind</t>
-  </si>
-  <si>
-    <t>Klasse</t>
-  </si>
-  <si>
-    <t>Eltern2</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="39">
   <si>
     <t>Gezahlt</t>
   </si>
@@ -127,13 +115,40 @@
   </si>
   <si>
     <t>Sim Hadzh</t>
+  </si>
+  <si>
+    <t>Eltern 1 - Name</t>
+  </si>
+  <si>
+    <t>Eltern 1 - Emailadresse</t>
+  </si>
+  <si>
+    <t>In Klasse</t>
+  </si>
+  <si>
+    <t>Name Kind</t>
+  </si>
+  <si>
+    <t>Adri.Mali@test.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max.Musterman@test.com </t>
+  </si>
+  <si>
+    <t>Alb.Trif@test.com</t>
+  </si>
+  <si>
+    <t>Alex.Nikolov@mux.com</t>
+  </si>
+  <si>
+    <t>Aleks.Hadzh@pux.com</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -145,6 +160,14 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -179,16 +202,19 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Link" xfId="1" builtinId="8"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -482,42 +508,42 @@
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" t="s">
-        <v>23</v>
+        <v>4</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>34</v>
       </c>
       <c r="E2">
         <v>530</v>
@@ -528,16 +554,16 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="B3" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" t="s">
-        <v>23</v>
+        <v>5</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>34</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -548,120 +574,120 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" t="s">
-        <v>26</v>
+        <v>6</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="E4">
         <v>540</v>
       </c>
       <c r="F4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="G4">
         <v>1</v>
       </c>
       <c r="H4" t="s">
-        <v>12</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" t="s">
-        <v>27</v>
+        <v>10</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>36</v>
       </c>
       <c r="E5">
         <v>360</v>
       </c>
       <c r="F5" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="G5">
         <v>1</v>
       </c>
       <c r="H5" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B6" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C6" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" t="s">
-        <v>29</v>
+        <v>13</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>37</v>
       </c>
       <c r="E6">
         <v>530</v>
       </c>
       <c r="F6" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="G6">
         <v>1</v>
       </c>
       <c r="H6" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B7" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C7" t="s">
-        <v>21</v>
-      </c>
-      <c r="D7" t="s">
-        <v>29</v>
+        <v>17</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>37</v>
       </c>
       <c r="E7">
         <v>530</v>
       </c>
       <c r="F7" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="G7">
         <v>1</v>
       </c>
       <c r="H7" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B8" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C8" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8" t="s">
-        <v>31</v>
+        <v>18</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="E8">
         <v>530</v>
@@ -672,16 +698,16 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B9" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="C9" t="s">
-        <v>22</v>
-      </c>
-      <c r="D9" t="s">
-        <v>31</v>
+        <v>18</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="E9">
         <v>0</v>
@@ -691,20 +717,28 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{190B1BF3-C3EB-4BA4-929C-F78A33405787}"/>
+    <hyperlink ref="D3" r:id="rId2" xr:uid="{676B47CB-19E5-4ACB-83D5-9A10C1A381AF}"/>
+    <hyperlink ref="D4" r:id="rId3" xr:uid="{531DEEC6-D44D-4746-90A9-0191EEE118EE}"/>
+    <hyperlink ref="D5" r:id="rId4" xr:uid="{9179C067-F531-4BEB-A85C-DBE924A2353E}"/>
+    <hyperlink ref="D6" r:id="rId5" xr:uid="{EA26D2F2-A574-4CE2-8D61-5BF4038E65BC}"/>
+    <hyperlink ref="D7" r:id="rId6" xr:uid="{75BD83FE-7D68-4C3D-83CD-68B2BC1EDFC1}"/>
+    <hyperlink ref="D8" r:id="rId7" xr:uid="{54907AF7-4E95-4E06-9477-7E86411D931C}"/>
+    <hyperlink ref="D9" r:id="rId8" xr:uid="{0AC92320-DD55-4983-8FC5-02084C8D756E}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId9"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="69b70055-4ccd-41e5-ba44-04aa7b40ef87">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="0d7d4427-3d9a-4210-88a6-80411ae356c7" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -903,21 +937,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="69b70055-4ccd-41e5-ba44-04aa7b40ef87">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="0d7d4427-3d9a-4210-88a6-80411ae356c7" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E6E074D9-8A3F-4B12-8FF2-84C884A0412A}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A75E2A0C-A03D-4EF1-AA2F-BC86D3F36961}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="69b70055-4ccd-41e5-ba44-04aa7b40ef87"/>
-    <ds:schemaRef ds:uri="0d7d4427-3d9a-4210-88a6-80411ae356c7"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -942,9 +975,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A75E2A0C-A03D-4EF1-AA2F-BC86D3F36961}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E6E074D9-8A3F-4B12-8FF2-84C884A0412A}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="69b70055-4ccd-41e5-ba44-04aa7b40ef87"/>
+    <ds:schemaRef ds:uri="0d7d4427-3d9a-4210-88a6-80411ae356c7"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>